<commit_message>
Template model, SVG card renderer, grid view and English UI with Italian translation
- Layer types (text, image, shape, group) with defaults and normalization
- Binding of sheet rows to templates: primary value and layer.property columns, {field} substitution
- Asset name resolution without path or extension, served through a gc-asset:// protocol
- SVG renderer in millimetres with text fit, image tint and flips, shapes and groups
- Set view with table or grid and a front/back preview of the selected card
- UI strings in English with Italian translation; load and binding messages travel as keys
- Demo project with real templates and placeholder art; vitest tests for binding and assets

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdURuMUp9T1LKbdt9ruT5G
</commit_message>
<xml_diff>
--- a/examples/demo/data/carte.xlsx
+++ b/examples/demo/data/carte.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
   <si>
     <t>amount</t>
   </si>
@@ -20,58 +20,97 @@
     <t>nome</t>
   </si>
   <si>
+    <t>banda</t>
+  </si>
+  <si>
     <t>forza</t>
   </si>
   <si>
     <t>testo</t>
   </si>
   <si>
-    <t>nome.color</t>
+    <t>forza_bg</t>
   </si>
   <si>
     <t>Cavaliere</t>
   </si>
   <si>
+    <t>#2F5DA8</t>
+  </si>
+  <si>
     <t>Quando attacchi, pesca una carta.</t>
   </si>
   <si>
-    <t>#1A56E8FF</t>
+    <t/>
   </si>
   <si>
     <t>Arciere</t>
   </si>
   <si>
-    <t>Può colpire a distanza.</t>
-  </si>
-  <si>
-    <t/>
+    <t>#3C7A3E</t>
+  </si>
+  <si>
+    <t>Può colpire un nemico a distanza 2.</t>
   </si>
   <si>
     <t>Strega</t>
   </si>
   <si>
-    <t>Scambia due carte sul tavolo.</t>
-  </si>
-  <si>
-    <t>#A706CCFF</t>
+    <t>#7A3FA0</t>
+  </si>
+  <si>
+    <t>Scambia due carte sul tavolo. Se una delle due è un Cavaliere, la Strega guadagna forza {forza} fino a fine turno.</t>
+  </si>
+  <si>
+    <t>Drago</t>
+  </si>
+  <si>
+    <t>#A33A2A</t>
+  </si>
+  <si>
+    <t>Non può essere bersaglio di magie.</t>
+  </si>
+  <si>
+    <t>#1A1A1A</t>
   </si>
   <si>
     <t>costo</t>
   </si>
   <si>
+    <t>icona</t>
+  </si>
+  <si>
+    <t>icona.tint</t>
+  </si>
+  <si>
     <t>effetto</t>
   </si>
   <si>
     <t>Pozione</t>
   </si>
   <si>
+    <t>pozione</t>
+  </si>
+  <si>
     <t>Recupera 2 punti vita.</t>
   </si>
   <si>
     <t>Spada</t>
   </si>
   <si>
+    <t>spada</t>
+  </si>
+  <si>
     <t>+2 forza.</t>
+  </si>
+  <si>
+    <t>Scudo</t>
+  </si>
+  <si>
+    <t>scudo</t>
+  </si>
+  <si>
+    <t>Annulla il prossimo attacco.</t>
   </si>
 </sst>
 </file>
@@ -448,10 +487,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -467,56 +506,88 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
       <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -527,10 +598,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -538,38 +609,76 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Text markup: Markdown, attributes, inline boxes, icons and styles
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DdYMc1KYPnMESWpVVXkVbH
</commit_message>
<xml_diff>
--- a/examples/demo/data/carte.xlsx
+++ b/examples/demo/data/carte.xlsx
@@ -38,7 +38,8 @@
     <t>#2F5DA8</t>
   </si>
   <si>
-    <t>Quando attacchi, pesca una carta.</t>
+    <t xml:space="preserve">Quando attacchi, pesca **una carta**.
+{.flavor} Il castello non cadrà stanotte.</t>
   </si>
   <si>
     <t/>
@@ -50,7 +51,7 @@
     <t>#3C7A3E</t>
   </si>
   <si>
-    <t>Può colpire un nemico a distanza 2.</t>
+    <t>Può colpire un [nemico]{.keyword} a distanza [2]{bg=circle bg-color=#3C7A3E color=white weight=800}.</t>
   </si>
   <si>
     <t>Strega</t>
@@ -59,7 +60,9 @@
     <t>#7A3FA0</t>
   </si>
   <si>
-    <t>Scambia due carte sul tavolo. Se una delle due è un Cavaliere, la Strega guadagna forza {forza} fino a fine turno.</t>
+    <t xml:space="preserve">Scambia due carte sul tavolo.
+- Se una è un [Cavaliere]{.keyword}, guadagna {spada*forza}
+- Altrimenti [Rapida]{border=#7A3FA0/0.3 radius=round color=#7A3FA0} fino a fine turno.</t>
   </si>
   <si>
     <t>Drago</t>
@@ -68,7 +71,10 @@
     <t>#A33A2A</t>
   </si>
   <si>
-    <t>Non può essere bersaglio di magie.</t>
+    <t xml:space="preserve"># Immune
+Non può essere bersaglio di ==magie==.
+---
+[Fuoco]{stroke=#A33A2A/12% color=#FFD27A size=+3 weight=900}</t>
   </si>
   <si>
     <t>#1A1A1A</t>
@@ -92,7 +98,7 @@
     <t>pozione</t>
   </si>
   <si>
-    <t>Recupera 2 punti vita.</t>
+    <t>Recupera [2]{bg=hexagon bg-color=#3C7A3E color=white weight=800} punti vita {pozione}.</t>
   </si>
   <si>
     <t>Spada</t>

</xml_diff>